<commit_message>
Replace template: Bill To → Company label in Excel
https://claude.ai/code/session_01QDisedv4fY96naKxX9qgHC
</commit_message>
<xml_diff>
--- a/CleanPotal/Resources/quotation_template.xlsx
+++ b/CleanPotal/Resources/quotation_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owner\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owner\source\repos\popo222kr-del\CleanPotal\CleanPotal\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60CE2972-5270-48B8-8F52-3EE94E020F76}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B73F96A-F4EE-46B5-B8DF-CB4F3DB08A34}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="330" windowWidth="12120" windowHeight="8700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -109,10 +109,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">	Bill To</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve">	Attention</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -130,6 +126,10 @@
   </si>
   <si>
     <t xml:space="preserve">	Biz. No.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">	Company</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -688,18 +688,8 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="179" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -723,9 +713,19 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="쉼표 [0]" xfId="1" builtinId="6"/>
@@ -1546,20 +1546,20 @@
       <c r="K9" s="6"/>
     </row>
     <row r="10" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="62" t="s">
+      <c r="A10" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="62"/>
-      <c r="C10" s="62"/>
-      <c r="D10" s="62"/>
-      <c r="E10" s="62"/>
-      <c r="F10" s="62"/>
-      <c r="G10" s="62"/>
-      <c r="H10" s="62"/>
-      <c r="I10" s="62"/>
-      <c r="J10" s="62"/>
-      <c r="K10" s="62"/>
-      <c r="L10" s="62"/>
+      <c r="B10" s="58"/>
+      <c r="C10" s="58"/>
+      <c r="D10" s="58"/>
+      <c r="E10" s="58"/>
+      <c r="F10" s="58"/>
+      <c r="G10" s="58"/>
+      <c r="H10" s="58"/>
+      <c r="I10" s="58"/>
+      <c r="J10" s="58"/>
+      <c r="K10" s="58"/>
+      <c r="L10" s="58"/>
     </row>
     <row r="11" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="H11" s="1"/>
@@ -1569,15 +1569,15 @@
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="70" t="s">
+      <c r="D12" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="70"/>
-      <c r="F12" s="70"/>
-      <c r="G12" s="70"/>
+      <c r="E12" s="57"/>
+      <c r="F12" s="57"/>
+      <c r="G12" s="57"/>
       <c r="H12" s="9"/>
       <c r="J12" s="56" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>14</v>
@@ -1587,16 +1587,16 @@
       <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="70" t="s">
+      <c r="D13" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="70"/>
-      <c r="F13" s="70"/>
-      <c r="G13" s="70"/>
+      <c r="E13" s="57"/>
+      <c r="F13" s="57"/>
+      <c r="G13" s="57"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="56" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>14</v>
@@ -1605,7 +1605,7 @@
     </row>
     <row r="14" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -1618,17 +1618,17 @@
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="56" t="s">
-        <v>25</v>
-      </c>
-      <c r="K14" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="K14" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="L14" s="57"/>
-      <c r="M14" s="58"/>
+      <c r="L14" s="69"/>
+      <c r="M14" s="70"/>
     </row>
     <row r="15" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -1643,11 +1643,11 @@
       <c r="J15" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="57" t="s">
+      <c r="K15" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="L15" s="57"/>
-      <c r="M15" s="58"/>
+      <c r="L15" s="69"/>
+      <c r="M15" s="70"/>
     </row>
     <row r="16" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="56" t="s">
@@ -1664,7 +1664,7 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="56" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K16" s="1" t="s">
         <v>14</v>
@@ -1714,13 +1714,13 @@
     </row>
     <row r="20" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="28"/>
-      <c r="B20" s="59"/>
-      <c r="C20" s="60"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
-      <c r="G20" s="60"/>
-      <c r="H20" s="61"/>
+      <c r="B20" s="66"/>
+      <c r="C20" s="67"/>
+      <c r="D20" s="67"/>
+      <c r="E20" s="67"/>
+      <c r="F20" s="67"/>
+      <c r="G20" s="67"/>
+      <c r="H20" s="68"/>
       <c r="I20" s="29"/>
       <c r="J20" s="30"/>
       <c r="K20" s="31"/>
@@ -1730,13 +1730,13 @@
     </row>
     <row r="21" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="28"/>
-      <c r="B21" s="59"/>
-      <c r="C21" s="60"/>
-      <c r="D21" s="60"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="60"/>
-      <c r="H21" s="61"/>
+      <c r="B21" s="66"/>
+      <c r="C21" s="67"/>
+      <c r="D21" s="67"/>
+      <c r="E21" s="67"/>
+      <c r="F21" s="67"/>
+      <c r="G21" s="67"/>
+      <c r="H21" s="68"/>
       <c r="I21" s="29"/>
       <c r="J21" s="30"/>
       <c r="K21" s="31"/>
@@ -1746,13 +1746,13 @@
     </row>
     <row r="22" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="28"/>
-      <c r="B22" s="59"/>
-      <c r="C22" s="60"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="60"/>
-      <c r="G22" s="60"/>
-      <c r="H22" s="61"/>
+      <c r="B22" s="66"/>
+      <c r="C22" s="67"/>
+      <c r="D22" s="67"/>
+      <c r="E22" s="67"/>
+      <c r="F22" s="67"/>
+      <c r="G22" s="67"/>
+      <c r="H22" s="68"/>
       <c r="I22" s="29"/>
       <c r="J22" s="30"/>
       <c r="K22" s="31"/>
@@ -1762,13 +1762,13 @@
     </row>
     <row r="23" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="28"/>
-      <c r="B23" s="59"/>
-      <c r="C23" s="60"/>
-      <c r="D23" s="60"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="60"/>
-      <c r="G23" s="60"/>
-      <c r="H23" s="61"/>
+      <c r="B23" s="66"/>
+      <c r="C23" s="67"/>
+      <c r="D23" s="67"/>
+      <c r="E23" s="67"/>
+      <c r="F23" s="67"/>
+      <c r="G23" s="67"/>
+      <c r="H23" s="68"/>
       <c r="I23" s="29"/>
       <c r="J23" s="30"/>
       <c r="K23" s="31"/>
@@ -1778,13 +1778,13 @@
     </row>
     <row r="24" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="28"/>
-      <c r="B24" s="59"/>
-      <c r="C24" s="60"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
-      <c r="G24" s="60"/>
-      <c r="H24" s="61"/>
+      <c r="B24" s="66"/>
+      <c r="C24" s="67"/>
+      <c r="D24" s="67"/>
+      <c r="E24" s="67"/>
+      <c r="F24" s="67"/>
+      <c r="G24" s="67"/>
+      <c r="H24" s="68"/>
       <c r="I24" s="29"/>
       <c r="J24" s="30"/>
       <c r="K24" s="31"/>
@@ -1794,13 +1794,13 @@
     </row>
     <row r="25" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="28"/>
-      <c r="B25" s="59"/>
-      <c r="C25" s="60"/>
-      <c r="D25" s="60"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="60"/>
-      <c r="G25" s="60"/>
-      <c r="H25" s="61"/>
+      <c r="B25" s="66"/>
+      <c r="C25" s="67"/>
+      <c r="D25" s="67"/>
+      <c r="E25" s="67"/>
+      <c r="F25" s="67"/>
+      <c r="G25" s="67"/>
+      <c r="H25" s="68"/>
       <c r="I25" s="29"/>
       <c r="J25" s="30"/>
       <c r="K25" s="31"/>
@@ -1810,13 +1810,13 @@
     </row>
     <row r="26" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="28"/>
-      <c r="B26" s="59"/>
-      <c r="C26" s="60"/>
-      <c r="D26" s="60"/>
-      <c r="E26" s="60"/>
-      <c r="F26" s="60"/>
-      <c r="G26" s="60"/>
-      <c r="H26" s="61"/>
+      <c r="B26" s="66"/>
+      <c r="C26" s="67"/>
+      <c r="D26" s="67"/>
+      <c r="E26" s="67"/>
+      <c r="F26" s="67"/>
+      <c r="G26" s="67"/>
+      <c r="H26" s="68"/>
       <c r="I26" s="29"/>
       <c r="J26" s="30"/>
       <c r="K26" s="31"/>
@@ -1826,13 +1826,13 @@
     </row>
     <row r="27" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="28"/>
-      <c r="B27" s="59"/>
-      <c r="C27" s="60"/>
-      <c r="D27" s="60"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="60"/>
-      <c r="G27" s="60"/>
-      <c r="H27" s="61"/>
+      <c r="B27" s="66"/>
+      <c r="C27" s="67"/>
+      <c r="D27" s="67"/>
+      <c r="E27" s="67"/>
+      <c r="F27" s="67"/>
+      <c r="G27" s="67"/>
+      <c r="H27" s="68"/>
       <c r="I27" s="29"/>
       <c r="J27" s="30"/>
       <c r="K27" s="31"/>
@@ -1842,13 +1842,13 @@
     </row>
     <row r="28" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="28"/>
-      <c r="B28" s="59"/>
-      <c r="C28" s="60"/>
-      <c r="D28" s="60"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="60"/>
-      <c r="G28" s="60"/>
-      <c r="H28" s="61"/>
+      <c r="B28" s="66"/>
+      <c r="C28" s="67"/>
+      <c r="D28" s="67"/>
+      <c r="E28" s="67"/>
+      <c r="F28" s="67"/>
+      <c r="G28" s="67"/>
+      <c r="H28" s="68"/>
       <c r="I28" s="29"/>
       <c r="J28" s="30"/>
       <c r="K28" s="31"/>
@@ -1858,13 +1858,13 @@
     </row>
     <row r="29" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="28"/>
-      <c r="B29" s="59"/>
-      <c r="C29" s="60"/>
-      <c r="D29" s="60"/>
-      <c r="E29" s="60"/>
-      <c r="F29" s="60"/>
-      <c r="G29" s="60"/>
-      <c r="H29" s="61"/>
+      <c r="B29" s="66"/>
+      <c r="C29" s="67"/>
+      <c r="D29" s="67"/>
+      <c r="E29" s="67"/>
+      <c r="F29" s="67"/>
+      <c r="G29" s="67"/>
+      <c r="H29" s="68"/>
       <c r="I29" s="29"/>
       <c r="J29" s="30"/>
       <c r="K29" s="31"/>
@@ -1874,13 +1874,13 @@
     </row>
     <row r="30" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="28"/>
-      <c r="B30" s="59"/>
-      <c r="C30" s="60"/>
-      <c r="D30" s="60"/>
-      <c r="E30" s="60"/>
-      <c r="F30" s="60"/>
-      <c r="G30" s="60"/>
-      <c r="H30" s="61"/>
+      <c r="B30" s="66"/>
+      <c r="C30" s="67"/>
+      <c r="D30" s="67"/>
+      <c r="E30" s="67"/>
+      <c r="F30" s="67"/>
+      <c r="G30" s="67"/>
+      <c r="H30" s="68"/>
       <c r="I30" s="29"/>
       <c r="J30" s="30"/>
       <c r="K30" s="31"/>
@@ -1890,13 +1890,13 @@
     </row>
     <row r="31" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="28"/>
-      <c r="B31" s="59"/>
-      <c r="C31" s="60"/>
-      <c r="D31" s="60"/>
-      <c r="E31" s="60"/>
-      <c r="F31" s="60"/>
-      <c r="G31" s="60"/>
-      <c r="H31" s="61"/>
+      <c r="B31" s="66"/>
+      <c r="C31" s="67"/>
+      <c r="D31" s="67"/>
+      <c r="E31" s="67"/>
+      <c r="F31" s="67"/>
+      <c r="G31" s="67"/>
+      <c r="H31" s="68"/>
       <c r="I31" s="29"/>
       <c r="J31" s="30"/>
       <c r="K31" s="31"/>
@@ -1954,13 +1954,13 @@
     </row>
     <row r="35" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="38"/>
-      <c r="B35" s="59"/>
-      <c r="C35" s="60"/>
-      <c r="D35" s="60"/>
-      <c r="E35" s="60"/>
-      <c r="F35" s="60"/>
-      <c r="G35" s="60"/>
-      <c r="H35" s="61"/>
+      <c r="B35" s="66"/>
+      <c r="C35" s="67"/>
+      <c r="D35" s="67"/>
+      <c r="E35" s="67"/>
+      <c r="F35" s="67"/>
+      <c r="G35" s="67"/>
+      <c r="H35" s="68"/>
       <c r="I35" s="30"/>
       <c r="J35" s="30"/>
       <c r="K35" s="31"/>
@@ -1970,13 +1970,13 @@
     </row>
     <row r="36" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="38"/>
-      <c r="B36" s="59"/>
-      <c r="C36" s="60"/>
-      <c r="D36" s="60"/>
-      <c r="E36" s="60"/>
-      <c r="F36" s="60"/>
-      <c r="G36" s="60"/>
-      <c r="H36" s="61"/>
+      <c r="B36" s="66"/>
+      <c r="C36" s="67"/>
+      <c r="D36" s="67"/>
+      <c r="E36" s="67"/>
+      <c r="F36" s="67"/>
+      <c r="G36" s="67"/>
+      <c r="H36" s="68"/>
       <c r="I36" s="30"/>
       <c r="J36" s="30"/>
       <c r="K36" s="31"/>
@@ -1986,13 +1986,13 @@
     </row>
     <row r="37" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="38"/>
-      <c r="B37" s="59"/>
-      <c r="C37" s="60"/>
-      <c r="D37" s="60"/>
-      <c r="E37" s="60"/>
-      <c r="F37" s="60"/>
-      <c r="G37" s="60"/>
-      <c r="H37" s="61"/>
+      <c r="B37" s="66"/>
+      <c r="C37" s="67"/>
+      <c r="D37" s="67"/>
+      <c r="E37" s="67"/>
+      <c r="F37" s="67"/>
+      <c r="G37" s="67"/>
+      <c r="H37" s="68"/>
       <c r="I37" s="30"/>
       <c r="J37" s="30"/>
       <c r="K37" s="31"/>
@@ -2002,13 +2002,13 @@
     </row>
     <row r="38" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="38"/>
-      <c r="B38" s="59"/>
-      <c r="C38" s="60"/>
-      <c r="D38" s="60"/>
-      <c r="E38" s="60"/>
-      <c r="F38" s="60"/>
-      <c r="G38" s="60"/>
-      <c r="H38" s="61"/>
+      <c r="B38" s="66"/>
+      <c r="C38" s="67"/>
+      <c r="D38" s="67"/>
+      <c r="E38" s="67"/>
+      <c r="F38" s="67"/>
+      <c r="G38" s="67"/>
+      <c r="H38" s="68"/>
       <c r="I38" s="30"/>
       <c r="J38" s="30"/>
       <c r="K38" s="31"/>
@@ -2018,13 +2018,13 @@
     </row>
     <row r="39" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="38"/>
-      <c r="B39" s="59"/>
-      <c r="C39" s="60"/>
-      <c r="D39" s="60"/>
-      <c r="E39" s="60"/>
-      <c r="F39" s="60"/>
-      <c r="G39" s="60"/>
-      <c r="H39" s="61"/>
+      <c r="B39" s="66"/>
+      <c r="C39" s="67"/>
+      <c r="D39" s="67"/>
+      <c r="E39" s="67"/>
+      <c r="F39" s="67"/>
+      <c r="G39" s="67"/>
+      <c r="H39" s="68"/>
       <c r="I39" s="30"/>
       <c r="J39" s="30"/>
       <c r="K39" s="31"/>
@@ -2034,13 +2034,13 @@
     </row>
     <row r="40" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="38"/>
-      <c r="B40" s="59"/>
-      <c r="C40" s="60"/>
-      <c r="D40" s="60"/>
-      <c r="E40" s="60"/>
-      <c r="F40" s="60"/>
-      <c r="G40" s="60"/>
-      <c r="H40" s="61"/>
+      <c r="B40" s="66"/>
+      <c r="C40" s="67"/>
+      <c r="D40" s="67"/>
+      <c r="E40" s="67"/>
+      <c r="F40" s="67"/>
+      <c r="G40" s="67"/>
+      <c r="H40" s="68"/>
       <c r="I40" s="30"/>
       <c r="J40" s="30"/>
       <c r="K40" s="31"/>
@@ -2050,13 +2050,13 @@
     </row>
     <row r="41" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="38"/>
-      <c r="B41" s="59"/>
-      <c r="C41" s="60"/>
-      <c r="D41" s="60"/>
-      <c r="E41" s="60"/>
-      <c r="F41" s="60"/>
-      <c r="G41" s="60"/>
-      <c r="H41" s="61"/>
+      <c r="B41" s="66"/>
+      <c r="C41" s="67"/>
+      <c r="D41" s="67"/>
+      <c r="E41" s="67"/>
+      <c r="F41" s="67"/>
+      <c r="G41" s="67"/>
+      <c r="H41" s="68"/>
       <c r="I41" s="40"/>
       <c r="J41" s="41"/>
       <c r="K41" s="42"/>
@@ -2065,31 +2065,31 @@
     </row>
     <row r="42" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="44"/>
-      <c r="B42" s="59"/>
-      <c r="C42" s="60"/>
-      <c r="D42" s="60"/>
-      <c r="E42" s="60"/>
-      <c r="F42" s="60"/>
-      <c r="G42" s="60"/>
-      <c r="H42" s="61"/>
+      <c r="B42" s="66"/>
+      <c r="C42" s="67"/>
+      <c r="D42" s="67"/>
+      <c r="E42" s="67"/>
+      <c r="F42" s="67"/>
+      <c r="G42" s="67"/>
+      <c r="H42" s="68"/>
       <c r="I42" s="45"/>
       <c r="J42" s="46"/>
       <c r="K42" s="47"/>
       <c r="L42" s="48"/>
     </row>
     <row r="43" spans="1:15" ht="17.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="67" t="s">
+      <c r="A43" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="68"/>
-      <c r="C43" s="68"/>
-      <c r="D43" s="68"/>
-      <c r="E43" s="68"/>
-      <c r="F43" s="68"/>
-      <c r="G43" s="68"/>
-      <c r="H43" s="68"/>
-      <c r="I43" s="68"/>
-      <c r="J43" s="69"/>
+      <c r="B43" s="64"/>
+      <c r="C43" s="64"/>
+      <c r="D43" s="64"/>
+      <c r="E43" s="64"/>
+      <c r="F43" s="64"/>
+      <c r="G43" s="64"/>
+      <c r="H43" s="64"/>
+      <c r="I43" s="64"/>
+      <c r="J43" s="65"/>
       <c r="K43" s="49">
         <f>SUM(K20:K42)</f>
         <v>0</v>
@@ -2202,11 +2202,11 @@
       <c r="L53" s="52"/>
     </row>
     <row r="55" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="J55" s="64" t="s">
+      <c r="J55" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="K55" s="65"/>
-      <c r="L55" s="65"/>
+      <c r="K55" s="61"/>
+      <c r="L55" s="61"/>
     </row>
     <row r="56" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="54"/>
@@ -2215,9 +2215,9 @@
       <c r="D56" s="54"/>
       <c r="E56" s="54"/>
       <c r="F56" s="54"/>
-      <c r="J56" s="66"/>
-      <c r="K56" s="66"/>
-      <c r="L56" s="66"/>
+      <c r="J56" s="62"/>
+      <c r="K56" s="62"/>
+      <c r="L56" s="62"/>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="J57" s="10" t="s">
@@ -2227,23 +2227,35 @@
       <c r="L57" s="55"/>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A59" s="63" t="s">
+      <c r="A59" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="B59" s="63"/>
-      <c r="C59" s="63"/>
-      <c r="D59" s="63"/>
-      <c r="E59" s="63"/>
-      <c r="F59" s="63"/>
-      <c r="G59" s="63"/>
-      <c r="H59" s="63"/>
-      <c r="I59" s="63"/>
-      <c r="J59" s="63"/>
-      <c r="K59" s="63"/>
-      <c r="L59" s="63"/>
+      <c r="B59" s="59"/>
+      <c r="C59" s="59"/>
+      <c r="D59" s="59"/>
+      <c r="E59" s="59"/>
+      <c r="F59" s="59"/>
+      <c r="G59" s="59"/>
+      <c r="H59" s="59"/>
+      <c r="I59" s="59"/>
+      <c r="J59" s="59"/>
+      <c r="K59" s="59"/>
+      <c r="L59" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="K14:M14"/>
+    <mergeCell ref="K15:M15"/>
+    <mergeCell ref="B30:H30"/>
+    <mergeCell ref="B31:H31"/>
+    <mergeCell ref="B40:H40"/>
+    <mergeCell ref="B41:H41"/>
+    <mergeCell ref="B42:H42"/>
+    <mergeCell ref="B35:H35"/>
+    <mergeCell ref="B36:H36"/>
+    <mergeCell ref="B37:H37"/>
+    <mergeCell ref="B38:H38"/>
+    <mergeCell ref="B39:H39"/>
     <mergeCell ref="D13:G13"/>
     <mergeCell ref="A10:L10"/>
     <mergeCell ref="A59:L59"/>
@@ -2260,18 +2272,6 @@
     <mergeCell ref="B28:H28"/>
     <mergeCell ref="B29:H29"/>
     <mergeCell ref="D12:G12"/>
-    <mergeCell ref="B41:H41"/>
-    <mergeCell ref="B42:H42"/>
-    <mergeCell ref="B35:H35"/>
-    <mergeCell ref="B36:H36"/>
-    <mergeCell ref="B37:H37"/>
-    <mergeCell ref="B38:H38"/>
-    <mergeCell ref="B39:H39"/>
-    <mergeCell ref="K14:M14"/>
-    <mergeCell ref="K15:M15"/>
-    <mergeCell ref="B30:H30"/>
-    <mergeCell ref="B31:H31"/>
-    <mergeCell ref="B40:H40"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
Fix broken layout for items 13-15 and 비고 lines in exported quotations
- The xlsx template was missing B32:H32/B33:H33/B34:H34 merge cell
  definitions (item rows 13-15), so longer Standard Spec/Description
  text in those rows wasn't merged across columns and got clipped
  against the Item-number column. Add the missing merge cells.
- Remark lines beyond the first (C46/C48/C50/C51) have no cell defined
  in the template, so newly created cells got the default style instead
  of matching C45's font/fill, making 비고 text look inconsistent.
  Force StyleIndex=1 on all 7 remark cells for consistent formatting.

https://claude.ai/code/session_01QDisedv4fY96naKxX9qgHC
</commit_message>
<xml_diff>
--- a/CleanPotal/Resources/quotation_template.xlsx
+++ b/CleanPotal/Resources/quotation_template.xlsx
@@ -2243,7 +2243,7 @@
       <c r="L59" s="59"/>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="31">
     <mergeCell ref="K14:M14"/>
     <mergeCell ref="K15:M15"/>
     <mergeCell ref="B30:H30"/>
@@ -2272,6 +2272,9 @@
     <mergeCell ref="B28:H28"/>
     <mergeCell ref="B29:H29"/>
     <mergeCell ref="D12:G12"/>
+    <mergeCell ref="B32:H32"/>
+    <mergeCell ref="B33:H33"/>
+    <mergeCell ref="B34:H34"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
Align item rows 13-15 cell styles with the rest of the item table
Even after merging B32:H32/B33:H33/B34:H34, those rows still used a
separate (but supposedly equivalent) style index for B-H than the
other item rows. Switch them to the exact same style indices used by
rows 20-31/35-42 so the bold Product Description formatting matches
across all item rows.

https://claude.ai/code/session_01QDisedv4fY96naKxX9qgHC
</commit_message>
<xml_diff>
--- a/CleanPotal/Resources/quotation_template.xlsx
+++ b/CleanPotal/Resources/quotation_template.xlsx
@@ -1906,13 +1906,13 @@
     </row>
     <row r="32" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="21"/>
-      <c r="B32" s="35"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="36"/>
-      <c r="E32" s="36"/>
-      <c r="F32" s="36"/>
-      <c r="G32" s="36"/>
-      <c r="H32" s="37"/>
+      <c r="B32" s="66"/>
+      <c r="C32" s="67"/>
+      <c r="D32" s="67"/>
+      <c r="E32" s="67"/>
+      <c r="F32" s="67"/>
+      <c r="G32" s="67"/>
+      <c r="H32" s="68"/>
       <c r="I32" s="30"/>
       <c r="J32" s="30"/>
       <c r="K32" s="31"/>
@@ -1922,13 +1922,13 @@
     </row>
     <row r="33" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="38"/>
-      <c r="B33" s="35"/>
-      <c r="C33" s="36"/>
-      <c r="D33" s="36"/>
-      <c r="E33" s="36"/>
-      <c r="F33" s="36"/>
-      <c r="G33" s="36"/>
-      <c r="H33" s="37"/>
+      <c r="B33" s="66"/>
+      <c r="C33" s="67"/>
+      <c r="D33" s="67"/>
+      <c r="E33" s="67"/>
+      <c r="F33" s="67"/>
+      <c r="G33" s="67"/>
+      <c r="H33" s="68"/>
       <c r="I33" s="30"/>
       <c r="J33" s="30"/>
       <c r="K33" s="31"/>
@@ -1938,13 +1938,13 @@
     </row>
     <row r="34" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="38"/>
-      <c r="B34" s="35"/>
-      <c r="C34" s="36"/>
-      <c r="D34" s="36"/>
-      <c r="E34" s="36"/>
-      <c r="F34" s="36"/>
-      <c r="G34" s="36"/>
-      <c r="H34" s="37"/>
+      <c r="B34" s="66"/>
+      <c r="C34" s="67"/>
+      <c r="D34" s="67"/>
+      <c r="E34" s="67"/>
+      <c r="F34" s="67"/>
+      <c r="G34" s="67"/>
+      <c r="H34" s="68"/>
       <c r="I34" s="30"/>
       <c r="J34" s="30"/>
       <c r="K34" s="31"/>

</xml_diff>

<commit_message>
Make item rows 14-21 number/amount columns bold to match rows above
A33-A40 and L33-L40 used non-bold cellXfs (38/39) while rows 20-32
used bold equivalents (21/32), causing item No. and Amount columns
for items 14-21 to render in a different (non-bold) font than the
rows above them.

https://claude.ai/code/session_01QDisedv4fY96naKxX9qgHC
</commit_message>
<xml_diff>
--- a/CleanPotal/Resources/quotation_template.xlsx
+++ b/CleanPotal/Resources/quotation_template.xlsx
@@ -1921,7 +1921,7 @@
       <c r="O32" s="34"/>
     </row>
     <row r="33" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="38"/>
+      <c r="A33" s="21"/>
       <c r="B33" s="66"/>
       <c r="C33" s="67"/>
       <c r="D33" s="67"/>
@@ -1932,12 +1932,12 @@
       <c r="I33" s="30"/>
       <c r="J33" s="30"/>
       <c r="K33" s="31"/>
-      <c r="L33" s="39"/>
+      <c r="L33" s="32"/>
       <c r="N33" s="33"/>
       <c r="O33" s="34"/>
     </row>
     <row r="34" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="38"/>
+      <c r="A34" s="21"/>
       <c r="B34" s="66"/>
       <c r="C34" s="67"/>
       <c r="D34" s="67"/>
@@ -1948,12 +1948,12 @@
       <c r="I34" s="30"/>
       <c r="J34" s="30"/>
       <c r="K34" s="31"/>
-      <c r="L34" s="39"/>
+      <c r="L34" s="32"/>
       <c r="N34" s="33"/>
       <c r="O34" s="34"/>
     </row>
     <row r="35" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="38"/>
+      <c r="A35" s="21"/>
       <c r="B35" s="66"/>
       <c r="C35" s="67"/>
       <c r="D35" s="67"/>
@@ -1964,12 +1964,12 @@
       <c r="I35" s="30"/>
       <c r="J35" s="30"/>
       <c r="K35" s="31"/>
-      <c r="L35" s="39"/>
+      <c r="L35" s="32"/>
       <c r="N35" s="33"/>
       <c r="O35" s="34"/>
     </row>
     <row r="36" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="38"/>
+      <c r="A36" s="21"/>
       <c r="B36" s="66"/>
       <c r="C36" s="67"/>
       <c r="D36" s="67"/>
@@ -1980,12 +1980,12 @@
       <c r="I36" s="30"/>
       <c r="J36" s="30"/>
       <c r="K36" s="31"/>
-      <c r="L36" s="39"/>
+      <c r="L36" s="32"/>
       <c r="N36" s="33"/>
       <c r="O36" s="34"/>
     </row>
     <row r="37" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="38"/>
+      <c r="A37" s="21"/>
       <c r="B37" s="66"/>
       <c r="C37" s="67"/>
       <c r="D37" s="67"/>
@@ -1996,12 +1996,12 @@
       <c r="I37" s="30"/>
       <c r="J37" s="30"/>
       <c r="K37" s="31"/>
-      <c r="L37" s="39"/>
+      <c r="L37" s="32"/>
       <c r="N37" s="33"/>
       <c r="O37" s="34"/>
     </row>
     <row r="38" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="38"/>
+      <c r="A38" s="21"/>
       <c r="B38" s="66"/>
       <c r="C38" s="67"/>
       <c r="D38" s="67"/>
@@ -2012,12 +2012,12 @@
       <c r="I38" s="30"/>
       <c r="J38" s="30"/>
       <c r="K38" s="31"/>
-      <c r="L38" s="39"/>
+      <c r="L38" s="32"/>
       <c r="N38" s="33"/>
       <c r="O38" s="34"/>
     </row>
     <row r="39" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="38"/>
+      <c r="A39" s="21"/>
       <c r="B39" s="66"/>
       <c r="C39" s="67"/>
       <c r="D39" s="67"/>
@@ -2028,12 +2028,12 @@
       <c r="I39" s="30"/>
       <c r="J39" s="30"/>
       <c r="K39" s="31"/>
-      <c r="L39" s="39"/>
+      <c r="L39" s="32"/>
       <c r="N39" s="33"/>
       <c r="O39" s="34"/>
     </row>
     <row r="40" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="38"/>
+      <c r="A40" s="21"/>
       <c r="B40" s="66"/>
       <c r="C40" s="67"/>
       <c r="D40" s="67"/>
@@ -2044,7 +2044,7 @@
       <c r="I40" s="30"/>
       <c r="J40" s="30"/>
       <c r="K40" s="31"/>
-      <c r="L40" s="39"/>
+      <c r="L40" s="32"/>
       <c r="N40" s="33"/>
       <c r="O40" s="34"/>
     </row>

</xml_diff>

<commit_message>
Make Standard Spec column bold for item rows 13-21
I32-I40 used non-bold cellXfs (30) while I20-I31 used a bold
equivalent (29), causing the Standard Spec (PartCode) column for
items 13-21 to render in a different (non-bold) font than the rows
above them.

https://claude.ai/code/session_01QDisedv4fY96naKxX9qgHC
</commit_message>
<xml_diff>
--- a/CleanPotal/Resources/quotation_template.xlsx
+++ b/CleanPotal/Resources/quotation_template.xlsx
@@ -1913,7 +1913,7 @@
       <c r="F32" s="67"/>
       <c r="G32" s="67"/>
       <c r="H32" s="68"/>
-      <c r="I32" s="30"/>
+      <c r="I32" s="35"/>
       <c r="J32" s="30"/>
       <c r="K32" s="31"/>
       <c r="L32" s="32"/>
@@ -1929,7 +1929,7 @@
       <c r="F33" s="67"/>
       <c r="G33" s="67"/>
       <c r="H33" s="68"/>
-      <c r="I33" s="30"/>
+      <c r="I33" s="35"/>
       <c r="J33" s="30"/>
       <c r="K33" s="31"/>
       <c r="L33" s="32"/>
@@ -1945,7 +1945,7 @@
       <c r="F34" s="67"/>
       <c r="G34" s="67"/>
       <c r="H34" s="68"/>
-      <c r="I34" s="30"/>
+      <c r="I34" s="35"/>
       <c r="J34" s="30"/>
       <c r="K34" s="31"/>
       <c r="L34" s="32"/>
@@ -1961,7 +1961,7 @@
       <c r="F35" s="67"/>
       <c r="G35" s="67"/>
       <c r="H35" s="68"/>
-      <c r="I35" s="30"/>
+      <c r="I35" s="35"/>
       <c r="J35" s="30"/>
       <c r="K35" s="31"/>
       <c r="L35" s="32"/>
@@ -1977,7 +1977,7 @@
       <c r="F36" s="67"/>
       <c r="G36" s="67"/>
       <c r="H36" s="68"/>
-      <c r="I36" s="30"/>
+      <c r="I36" s="35"/>
       <c r="J36" s="30"/>
       <c r="K36" s="31"/>
       <c r="L36" s="32"/>
@@ -1993,7 +1993,7 @@
       <c r="F37" s="67"/>
       <c r="G37" s="67"/>
       <c r="H37" s="68"/>
-      <c r="I37" s="30"/>
+      <c r="I37" s="35"/>
       <c r="J37" s="30"/>
       <c r="K37" s="31"/>
       <c r="L37" s="32"/>
@@ -2009,7 +2009,7 @@
       <c r="F38" s="67"/>
       <c r="G38" s="67"/>
       <c r="H38" s="68"/>
-      <c r="I38" s="30"/>
+      <c r="I38" s="35"/>
       <c r="J38" s="30"/>
       <c r="K38" s="31"/>
       <c r="L38" s="32"/>
@@ -2025,7 +2025,7 @@
       <c r="F39" s="67"/>
       <c r="G39" s="67"/>
       <c r="H39" s="68"/>
-      <c r="I39" s="30"/>
+      <c r="I39" s="35"/>
       <c r="J39" s="30"/>
       <c r="K39" s="31"/>
       <c r="L39" s="32"/>
@@ -2041,7 +2041,7 @@
       <c r="F40" s="67"/>
       <c r="G40" s="67"/>
       <c r="H40" s="68"/>
-      <c r="I40" s="30"/>
+      <c r="I40" s="35"/>
       <c r="J40" s="30"/>
       <c r="K40" s="31"/>
       <c r="L40" s="32"/>

</xml_diff>